<commit_message>
Add Gemini provider support with pluggable AI layer
</commit_message>
<xml_diff>
--- a/data/internship_outreach.xlsx
+++ b/data/internship_outreach.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16840" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Companies" sheetId="1" state="visible" r:id="rId1"/>
@@ -18,14 +17,14 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Outreach'!$A$1:$T$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Settings'!$A$1:$B$1</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,9 +33,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -48,7 +57,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,17 +70,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -435,35 +447,21 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AA11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="4" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
     <col width="35" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="12" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="16" max="23"/>
     <col width="50" customWidth="1" min="24" max="24"/>
-    <col width="18" customWidth="1" min="25" max="25"/>
-    <col width="18" customWidth="1" min="26" max="26"/>
-    <col width="18" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="25" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -629,28 +627,65 @@
           <t>Nairobi</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Technology organisation (mock summary).</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Technology and data teams (mock summary).</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Mock evidence -- not a real finding.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.safaricom.co.ke/careers</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Data Analyst Intern; Software Intern</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>18</v>
+      </c>
+      <c r="R2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S2" t="n">
+        <v>9</v>
+      </c>
+      <c r="T2" t="n">
+        <v>8</v>
+      </c>
+      <c r="U2" t="n">
+        <v>9</v>
+      </c>
+      <c r="V2" t="n">
+        <v>83</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>[MOCK RESULT -- not a real assessment] Retrieved pages mention technology and hiring signals (9 indicators matched).</t>
+        </is>
+      </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>QUALIFY</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -690,28 +725,65 @@
           <t>Nairobi</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>5</v>
+      </c>
+      <c r="R3" t="n">
+        <v>10</v>
+      </c>
+      <c r="S3" t="n">
+        <v>5</v>
+      </c>
+      <c r="T3" t="n">
+        <v>3</v>
+      </c>
+      <c r="U3" t="n">
+        <v>9</v>
+      </c>
+      <c r="V3" t="n">
+        <v>44</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>[MOCK RESULT -- not a real assessment] No evidence could be retrieved, so no confident judgement is possible. This is a data gap, not a negative finding.</t>
+        </is>
+      </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>NEEDS_REVIEW</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -751,25 +823,6 @@
           <t>Nairobi</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr">
         <is>
           <t>PENDING</t>
@@ -812,25 +865,6 @@
           <t>Nairobi</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr">
         <is>
           <t>PENDING</t>
@@ -873,25 +907,6 @@
           <t>Nairobi</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr">
         <is>
           <t>PENDING</t>
@@ -934,25 +949,6 @@
           <t>Nairobi</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr">
         <is>
           <t>PENDING</t>
@@ -995,25 +991,6 @@
           <t>Nairobi</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr">
         <is>
           <t>PENDING</t>
@@ -1056,25 +1033,6 @@
           <t>Nairobi</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr">
         <is>
           <t>PENDING</t>
@@ -1117,25 +1075,6 @@
           <t>Nairobi</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr">
         <is>
           <t>PENDING</t>
@@ -1178,25 +1117,6 @@
           <t>Nairobi</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr">
         <is>
           <t>PENDING</t>
@@ -1226,14 +1146,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="4" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
@@ -1317,25 +1234,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:T1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="1" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="5" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="70" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="9" max="17"/>
     <col width="40" customWidth="1" min="18" max="18"/>
     <col width="25" customWidth="1" min="19" max="19"/>
     <col width="30" customWidth="1" min="20" max="20"/>
@@ -1456,7 +1362,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
@@ -1528,9 +1434,9 @@
           <t>Email</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>FILL_IN</t>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>monicawughanga@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1448,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FILL_IN</t>
+          <t>https://www.linkedin.com/in/monica-masae/</t>
         </is>
       </c>
     </row>
@@ -1552,9 +1458,9 @@
           <t>GitHub</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>FILL_IN</t>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/M0nicah</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1496,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FILL_IN</t>
+          <t>Immiediately</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1520,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FILL_IN</t>
+          <t>Nairobi</t>
         </is>
       </c>
     </row>
@@ -1644,6 +1550,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:B1"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Stage 3 verified: Gemini provider, retries, honest evidence-based qualification
</commit_message>
<xml_diff>
--- a/data/internship_outreach.xlsx
+++ b/data/internship_outreach.xlsx
@@ -629,17 +629,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Technology organisation (mock summary).</t>
+          <t>Safaricom PLC provides telecommunications, mobile money (M-PESA), internet, and digital services in Kenya.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Technology and data teams (mock summary).</t>
+          <t>Extensive telecommunications network infrastructure, mobile financial platforms (M-PESA), cloud solutions, and software development teams.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mock evidence -- not a real finding.</t>
+          <t>The careers page explicitly features an 'Internship Program' and references software engineers on staff.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -649,38 +649,38 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Data Analyst Intern; Software Intern</t>
+          <t>Data Analyst; Data Science Intern; Data/Research Assistant; Business Intelligence; Data Operations; Software/Web Development</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="Q2" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="R2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="S2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="U2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V2" t="n">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>[MOCK RESULT -- not a real assessment] Retrieved pages mention technology and hiring signals (9 indicators matched).</t>
+          <t>Safaricom PLC is a major telecommunications and digital services provider in Nairobi with an explicit Internship Program listed on its careers portal and a strong technical function including software engineering and digital services.</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -742,16 +742,16 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>https://equitygroupholdings.com/careers</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>Data Analyst; Data Science Intern; Business Intelligence; IT; Software/Web Development</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="Q3" t="n">
         <v>5</v>
@@ -760,25 +760,25 @@
         <v>10</v>
       </c>
       <c r="S3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="T3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V3" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>NEEDS_REVIEW</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>[MOCK RESULT -- not a real assessment] No evidence could be retrieved, so no confident judgement is possible. This is a data gap, not a negative finding.</t>
+          <t>The website requests to equitygroupholdings.com and its careers page were unsuccessful due to Incapsula security blocks, preventing verification of current technology functions and contact routes. However, as a major bank based in Nairobi, it likely has IT and data operations, making it a candidate for review once access is resolved.</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://twiga.com</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -823,9 +823,65 @@
           <t>Nairobi</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Data Analyst; Data Science Intern; Business Intelligence</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S4" t="n">
+        <v>5</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>10</v>
+      </c>
+      <c r="V4" t="n">
+        <v>35</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>NEEDS_REVIEW</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>No evidence retrieved or website recorded for this company, preventing any assessment of its technology function or contactability.</t>
+        </is>
+      </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>NEEDS_REVIEW</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -865,9 +921,65 @@
           <t>Nairobi</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Data Analyst; Data Science Intern; Software/Web Development</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>10</v>
+      </c>
+      <c r="S5" t="n">
+        <v>5</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
+        <v>10</v>
+      </c>
+      <c r="V5" t="n">
+        <v>35</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>NEEDS_REVIEW</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>The website access was blocked with an HTTP 403 error, resulting in no retrieved evidence. Per instructions, absence of evidence due to a blocked website requires a NEEDS_REVIEW response rather than a rejection, though the current score reflects the lack of verifiable data.</t>
+        </is>
+      </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>NEEDS_REVIEW</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
@@ -907,9 +1019,65 @@
           <t>Nairobi</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Data Science Intern; Data Analyst; Software/Web Development</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R6" t="n">
+        <v>10</v>
+      </c>
+      <c r="S6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>5</v>
+      </c>
+      <c r="V6" t="n">
+        <v>35</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>NEEDS_REVIEW</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>The evidence block states that access to the website was blocked by the website with an HTTP 403 error, resulting in no retrieved text or evidence about the organisation. Therefore, a confident decision cannot be made based on the provided evidence.</t>
+        </is>
+      </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>NEEDS_REVIEW</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
@@ -936,7 +1104,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://ilabafrica.ac.ke</t>
+          <t>https://ilabafrica.strathmore.edu</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -949,9 +1117,65 @@
           <t>Nairobi</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Strathmore University iLabAfrica is a research and innovation centre focusing on ICT development, artificial intelligence, and digital transformation.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Research, software development, data science, cybersecurity, and IoT projects.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Data Science Intern; Data Analyst; Data/Research Assistant; Software/Web Development Intern</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>15</v>
+      </c>
+      <c r="R7" t="n">
+        <v>20</v>
+      </c>
+      <c r="S7" t="n">
+        <v>10</v>
+      </c>
+      <c r="T7" t="n">
+        <v>8</v>
+      </c>
+      <c r="U7" t="n">
+        <v>10</v>
+      </c>
+      <c r="V7" t="n">
+        <v>88</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Strathmore University iLabAfrica is a dedicated research and innovation centre focusing on ICT, data science, artificial intelligence, and software development, providing an exceptional match for a BSc Data Science student based in Nairobi. While no explicit careers page was found in the text, the organisation hosts specific academic programmes, data science units, and technology research projects that align directly with the student's skills.</t>
+        </is>
+      </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>QUALIFY</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
@@ -991,9 +1215,65 @@
           <t>Nairobi</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="n">
+        <v>5</v>
+      </c>
+      <c r="V8" t="n">
+        <v>5</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>NEEDS_REVIEW</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>No evidence was retrieved because the website could not be connected. As a result, the technical function, maturity, and contactability could not be checked based on the provided data.</t>
+        </is>
+      </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>NEEDS_REVIEW</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
@@ -1033,9 +1313,65 @@
           <t>Nairobi</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>The decision rests on the name alone, as Jamii Cyber Cafe indicates a type of business focused on retail internet and typing services rather than professional technology, data, or software engineering functions.</t>
+        </is>
+      </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
@@ -1075,9 +1411,65 @@
           <t>Nairobi</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>The decision rests on the name alone, as 'Kilimani Computer Repairs' clearly and unambiguously identifies the business type as a computer repair shop rather than a professional software, data, or technology organisation suited for a BSc Data Science student.</t>
+        </is>
+      </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
@@ -1117,9 +1509,65 @@
           <t>Nairobi</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>The decision rests on the organisation's name alone, which clearly and unambiguously identifies it as a phone accessories retailer rather than a professional technology or data science organisation.</t>
+        </is>
+      </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">

</xml_diff>

<commit_message>
Stage 4: reporting. Stage 5: contact research with anti-fabrication guard
</commit_message>
<xml_diff>
--- a/data/internship_outreach.xlsx
+++ b/data/internship_outreach.xlsx
@@ -1593,7 +1593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="2"/>
@@ -1666,6 +1666,316 @@
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Contact Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Safaricom PLC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Careers / application portal</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Internship/Graduate Recruitment</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://www.safaricom.co.ke/careers</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>This is the official careers portal of Safaricom PLC intended for job and internship applications. (source: https://www.safaricom.co.ke/careers)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Safaricom PLC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>advantage@safaricom.co.ke</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>OBSERVED</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://www.safaricom.co.ke/careers</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>This address represents a product or service offering published on the careers page rather than a recruitment or HR inbox. (source: https://www.safaricom.co.ke/careers)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Safaricom PLC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>customercare@safaricom.co.ke</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>OBSERVED</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://www.safaricom.co.ke/careers</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>This is a customer support email address published on the careers page, which is not handled by hiring teams. (source: https://www.safaricom.co.ke/careers)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>C002</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Equity Bank Kenya</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Careers / application portal</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Internship/Graduate Recruitment</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://equitygroupholdings.com/careers</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>This route is the official careers portal published on the organisation's website. (source: https://equitygroupholdings.com/careers)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>C006</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Strathmore University iLabAfrica</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ilabafrica@strathmore.edu</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>OBSERVED</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://ilabafrica.strathmore.edu/</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>This is a general institutional and contact email address published on the homepage of Strathmore University iLabAfrica. (source: https://ilabafrica.strathmore.edu/)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>NEW</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stage 6: email drafting with grounded personalisation and quality checks
</commit_message>
<xml_diff>
--- a/data/internship_outreach.xlsx
+++ b/data/internship_outreach.xlsx
@@ -1991,7 +1991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="3"/>
@@ -2106,6 +2106,248 @@
           <t>Notes</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>O001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Safaricom PLC</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Campaign 2 - Software / Technology Internship</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - software and web development support</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Dear Safaricom PLC Team,
+I am Monica Wughanga Masae, a BSc Data Science student at the Open University of Kenya, graduating in 2027.
+I am writing to enquire about internship or industrial attachment opportunities relating to your software development teams and digital services.
+Through my studies and software projects, I have worked with Python, R, SQL, and web development. I can contribute to application support, data analysis, and technical documentation while building my practical skills in a professional environment.
+I would like to know if you currently consider students for an internship or industrial attachment placement, and who I should direct my application to if not the recipient of this email.
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>O002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>C002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P004</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Equity Bank Kenya</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Campaign 4 - General Technology Internship</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - data and technology support</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Dear Equity Bank Kenya Team,
+I am a student at the Open University of Kenya pursuing a BSc in Data Science, with an expected graduation year of 2027.
+I am writing to enquire about opportunities for an internship or industrial attachment involving data, IT, and general technology work.
+Through my studies and personal projects, I have built practical skills in Python, R, SQL, Excel, data analysis, visualization, and basic machine learning, alongside web development and technical reporting. I am looking to contribute these capabilities to your technical operations while gaining hands-on experience in a professional environment.
+Could you please let me know if you would consider an intern or industrial attachment placement, and if so, who the appropriate person is to speak with regarding this?
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>O003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>C006</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Strathmore University iLabAfrica</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Campaign 3 - AI / ML Internship</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - AI, ML and data science</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Dear Strathmore University iLabAfrica Team,
+I am a BSc Data Science student at the Open University of Kenya, graduating in 2027.
+I am writing to enquire about internship or industrial attachment opportunities at Strathmore University iLabAfrica, given your focus on ICT development, artificial intelligence, and digital transformation, as well as your work on research, software development, data science, cybersecurity, and IoT projects.
+Through my coursework, I have built skills in Python, R, SQL, data analysis, visualization, and basic machine learning, alongside experience in software projects and technical documentation. I am available immediately for an internship or industrial attachment placement in Nairobi, and I am eager to contribute to your data and technology operations while building on my foundational machine learning knowledge.
+Please let me know if you consider interns or industrial attachment students, and who I should direct my application to if you are the wrong contact.
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:T1"/>

</xml_diff>

<commit_message>
Stage 7: approval gate, manual send export and tracking
</commit_message>
<xml_diff>
--- a/data/internship_outreach.xlsx
+++ b/data/internship_outreach.xlsx
@@ -2174,19 +2174,11 @@
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2255,19 +2247,11 @@
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2322,12 +2306,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -2335,19 +2319,26 @@
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="P4" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Sent manually via Gmail Sent manually before approval; recorded with --force.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:T1"/>

</xml_diff>

<commit_message>
Fix duplicate drafting for already-contacted companies
</commit_message>
<xml_diff>
--- a/data/internship_outreach.xlsx
+++ b/data/internship_outreach.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16840" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4420" yWindow="660" windowWidth="24980" windowHeight="16840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Companies" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,10 +12,10 @@
     <sheet name="Settings" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Companies'!$A$1:$AA$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Contacts'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Outreach'!$A$1:$T$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Settings'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Companies'!$A$1:$AA$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Contacts'!$A$1:$L$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Outreach'!$A$1:$T$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Settings'!$A$1:$B$15</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,17 +446,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA44"/>
+  <dimension ref="A1:AA78"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="35" customWidth="1" min="10" max="10"/>
-    <col width="45" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="13"/>
+    <col width="18" customWidth="1" min="4" max="5"/>
+    <col width="35.5" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="8"/>
+    <col width="134.6640625" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="119.1640625" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="158.33203125" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="89.83203125" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="23"/>
@@ -4985,8 +4988,1606 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>C044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Leta</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://leta.ai</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>AI Logistics Software</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>Search: logistics technology company Nairobi</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>C045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>BETA Agriculture Technologies</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://www.betaagritech.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>AgriTech</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>Search: agritech data company Kenya</t>
+        </is>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>C046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>AgriKenya</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://agrikenya.co.ke</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Digital Solutions / AgriTech</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>Search: agritech data company Kenya</t>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>C047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>InsurTech Forum Nairobi</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://insurtechforum.insure</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Fintech / InsurTech</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>Search: insurtech Nairobi Kenya</t>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>C048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>bolttech</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://bolttech.io</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>InsurTech</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>Search: insurtech Nairobi Kenya</t>
+        </is>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>C049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>World Food Programme</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://wfp.org</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>UN agency / Humanitarian data</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>C050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>World Health Organization</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://who.int</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>UN agency / Health data</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>C051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>World Bank</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://worldbank.org</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>International finance / Development data</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>C052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Kenya Red Cross Society</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://redcross.or.ke</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Humanitarian / Emergency data systems</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>C053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Amref Health Africa</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://amref.org</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Health NGO / Health informatics</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>C054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>PATH</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://path.org</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Global health NGO / Health data</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z55" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>C055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Population Services International</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://psi.org</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Global health NGO / M&amp;E</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z56" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA56" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>C056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>CARE International</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://care.org</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Humanitarian NGO / M&amp;E</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z57" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>C057</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Oxfam</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://oxfam.org</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Humanitarian NGO / Research</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z58" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>C058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ActionAid</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://actionaid.org</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Development NGO / M&amp;E</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>C059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Mercy Corps</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://mercycorps.org</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Humanitarian NGO / Data and evidence</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>C060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ICT Authority Kenya</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://icta.go.ke</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Government / National ICT</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z61" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>C061</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Kenya National Bureau of Statistics</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://knbs.or.ke</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Government / Official statistics</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z62" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>C062</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Central Bank of Kenya</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://centralbank.go.ke</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Government / Financial data</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>C063</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Communications Authority of Kenya</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://cak.go.ke</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Government regulator / Telecom data</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z64" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>C064</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>National Hospital Insurance Fund</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://nhif.or.ke</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Government / Health insurance systems</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>C065</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>The National Treasury Kenya</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://treasury.go.ke</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Government / Public finance data</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>C066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Nairobi City County</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://nairobi.go.ke</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>County government / Public services data</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>C067</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Kenya National Highways Authority</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://kenha.co.ke</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Government agency / Infrastructure data</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z68" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>C068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>National Industrial Training Authority</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://nita.go.ke</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Government / Training and skills data</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>C069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Kenya Power</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://kplc.co.ke</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Utility / Energy data systems</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z70" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>C070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Wasoko</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://wasoko.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>B2B e-commerce startup / Logistics tech</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>C071</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Pezesha</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://pezesha.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Fintech startup / Embedded lending</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>C072</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>4G Capital</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://4g-capital.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Fintech / Micro-lending data</t>
+        </is>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z73" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA73" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>C073</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Turaco</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://turaco.insure</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Insurtech startup</t>
+        </is>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z74" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA74" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>C074</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Jumia Kenya</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://jumia.co.ke</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>E-commerce / Marketplace data</t>
+        </is>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA75" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>C075</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Little Cab</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://littlecab.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Ride-hailing / Mobility tech</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>C076</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Glovo</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://glovoapp.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Delivery platform / Logistics data</t>
+        </is>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z77" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA77" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>C077</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Bolt</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://bolt.eu</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Nairobi</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Ride-hailing / Mobility data</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>Curated sector list</t>
+        </is>
+      </c>
+      <c r="AA78" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA1"/>
+  <autoFilter ref="A1:AA78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7740,7 +9341,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:L44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7751,15 +9352,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T30"/>
+  <dimension ref="A1:T51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="6"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="36.6640625" bestFit="1" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="70" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="17"/>
+    <col width="15.6640625" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="12.83203125" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="13.5" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="15.33203125" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="17"/>
     <col width="40" customWidth="1" min="18" max="18"/>
     <col width="25" customWidth="1" min="19" max="19"/>
     <col width="30" customWidth="1" min="20" max="20"/>
@@ -9180,12 +10786,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>NOT_STARTED</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -9196,6 +10802,11 @@
       <c r="P19" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Duplicate of O004 - already applied via their careers portal.</t>
         </is>
       </c>
     </row>
@@ -9997,24 +11608,1545 @@
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
           <t>Logged manually: applied via their website with tailored CV and cover letter</t>
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>O030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>C043</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>P046</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Rudder Research and Data Analytics LTD</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Campaign 1 - Data / Analytics Internship</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Internship enquiry - data analysis and reporting, BSc Data Science student</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Dear Rudder Research and Data Analytics LTD Team,
+My name is Monica Wughanga Masae, and I am studying BSc Data Science at the Open University of Kenya, with an expected graduation in 2027.
+I am reaching out because your consultancy supports evidence-led decisions through research, data cleaning and analysis, dashboards, and reporting for companies, NGOs, and SACCOs working in Kenya.
+I can contribute practical skills in Python, R, SQL, Excel, data analysis, data visualization, and reporting from my studies and software projects. I want to build on these skills through hands-on work with survey design, field data collection, and data analysis.
+I am writing to ask whether you would consider a student for an internship or industrial attachment placement in Nairobi. If you do not currently host interns, please let me know the appropriate person to speak with regarding data analyst roles.
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>NOT_STARTED</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Duplicate of O029 - already applied via their website on 2026-09-14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>O031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>C048</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>P047</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>bolttech</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Campaign 2 - Software / Technology Internship</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - software and web development support</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Dear bolttech Team,
+I am Monica Wughanga Masae, a BSc Data Science student at the Open University of Kenya graduating in 2027.
+I am writing to enquire about internship or industrial attachment opportunities relating to your work in operating an international insurtech business providing a B2B2C protection and insurance platform, specifically regarding the development and maintenance of digital insurance distribution engines, embedded insurance APIs, data insights platforms, and no-code product configurators.
+Through my studies and personal projects, I have built practical skills in Python, SQL, web development, software projects, and technical documentation, and I am keen to apply and expand these abilities in application support and software development tasks.
+I would like to know if you would consider taking on an intern or industrial attachment student for this type of work, and if not, who the appropriate person to speak with would be.
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>O032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>C049</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>P048</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>World Food Programme</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Campaign 1 - Data / Analytics Internship</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Internship enquiry - data analysis, reporting and visualisation, BSc Data Science student</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Dear World Food Programme Team,
+I am a student at the Open University of Kenya pursuing a BSc in Data Science, with an expected graduation in 2027. I am writing to enquire about an internship or industrial attachment.
+I am interested in your work delivering food assistance and supporting sustainable livelihoods worldwide, specifically regarding your data analysis, reporting, and logistics systems supporting global humanitarian operations.
+Through my studies and personal projects, I have built practical skills in Python, R, SQL, Excel, data analysis, data visualization, and Tableau exposure. I am looking for an opportunity to contribute to data analysis, reporting, and visualisation work while learning from your team.
+I am available immediately in Nairobi and would like to know if you consider interns or industrial attachment students. If you are not the correct person to speak with regarding this, could you please direct me to the appropriate contact.
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>O033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>C050</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>P049</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>World Health Organization</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Campaign 1 - Data / Analytics Internship</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Internship enquiry - data analysis, BSc Data Science student</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Dear World Health Organization Team,
+My name is Monica Wughanga Masae, and I am studying for a BSc in Data Science at the Open University of Kenya, with an expected graduation in 2027.
+I am reaching out because you maintain extensive global health data and research operations, and handle data collection, global health estimates, statistical dashboards, and health information systems.
+I can contribute skills in data analysis, reporting, visualisation, Python, R, SQL, and Excel through my studies and projects. I want to learn more about applying these methods to public health data operations.
+Could you please consider me for an internship or industrial attachment placement in Nairobi, or let me know who I should speak with regarding such opportunities?
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>O034</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>C051</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>P050</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>World Bank</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Campaign 2 - Software / Technology Internship</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - software and web development support</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Dear World Bank Team,
+I am a BSc Data Science student at the Open University of Kenya, graduating in 2027, writing to enquire about an internship or industrial attachment.
+My studies focus on data collection, digital development initiatives, and information technology infrastructure supporting global operations.
+Through my coursework and personal projects, I have worked with Python, SQL, web development, and software projects, along with basic machine learning, data analysis, and reporting. I want to contribute these skills to your software and web development work while building practical experience in application support and technology operations.
+I would like to know if you consider students for internship or industrial attachment placements in this area, and who the appropriate person to contact would be if not you.
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>O035</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>C052</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>P051</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Kenya Red Cross Society</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Campaign 4 - General Technology Internship</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - data, IT, and general technology support</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Dear Kenya Red Cross Society Team,
+I am Monica Wughanga Masae, a BSc Data Science student at the Open University of Kenya, graduating in 2027.
+I am reaching out regarding potential opportunities for an internship or industrial attachment to support general technology, IT, and data work within your humanitarian relief operations.
+Through my studies and software projects, I have built practical skills in Python, R, SQL, Excel, data analysis, visualization, and basic machine learning, alongside exposure to Tableau and web development. I am eager to apply these technical abilities and learn from your team.
+Could you please let me know if you consider students for internships or industrial attachments, and who the appropriate person to contact would be if this falls outside your purview?
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>O036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>C053</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>P052</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Amref Health Africa</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Campaign 4 - General Technology Internship</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - technology, IT and data work</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Dear Amref Health Africa Team,
+I am a BSc Data Science student at the Open University of Kenya, with an expected graduation year of 2027.
+I am writing to enquire about potential internship or industrial attachment opportunities related to your technology function, which involves monitoring, evaluation, research publications, and digital health initiatives.
+Through my studies, I have built practical skills in Python, R, SQL, Excel, data analysis, data visualization, basic machine learning, and software projects. I am eager to apply these technical skills to support your data operations and technology work while further developing my capabilities.
+Could you please let me know if you consider students for internships or industrial attachments, and who the appropriate person is to contact regarding such opportunities?
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>O037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>C054</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>P054</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>PATH</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Campaign 4 - General Technology Internship</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - technology, IT and data work</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Dear PATH Team,
+I am Monica Wughanga Masae, a BSc Data Science student at the Open University of Kenya with an expected graduation year of 2027.
+I am writing to enquire about internship or industrial attachment opportunities relating to your technology, IT and data work.
+Through my studies and personal projects, I have built practical skills in Python, R, SQL, Excel, data analysis, visualization, basic machine learning, and software projects.
+I am seeking an internship or industrial attachment placement in Nairobi to apply these skills and learn from your team, and I am available to start immediately. If you do not currently host interns or attachments, could you let me know who might be appropriate to speak with regarding these opportunities.
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>O038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>C055</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>P056</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Population Services International</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Campaign 4 - General Technology Internship</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - data analysis and technology, BSc Data Science student</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Dear Population Services International Team,
+I am Monica Wughanga Masae, a BSc Data Science student at the Open University of Kenya, graduating in 2027.
+I am reaching out regarding potential opportunities because your work involves digital health projects and data management across global health initiatives.
+Through my studies and software projects, I have built practical skills in Python, R, SQL, Excel, data analysis, data visualization, basic machine learning, and technical documentation. I am available immediately for an internship or industrial attachment to support your technology function while learning from your team.
+Could you please let me know if you would consider a student placement, and who I might speak with if applications are handled elsewhere?
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>O039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>C056</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>P057</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>CARE International</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Campaign 2 - Software / Technology Internship</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - software and web development support</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Dear CARE International Team,
+I am Monica Wughanga Masae, a BSc Data Science student at the Open University of Kenya with an expected graduation year of 2027.
+I am writing to enquire about internship or industrial attachment opportunities. I note from your careers page that you feature a search for internships option, and I am interested in supporting the technology and operational functions involved in your humanitarian aid and development work.
+Through my studies and software projects, I have built skills in Python, SQL, web development, and software applications. I want to contribute to your software and web development or application support tasks while learning how data and technology are applied in an international organisation.
+Could you please let me know if you consider interns or industrial attachments, and who I should direct this enquiry to if you are not the correct contact?
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>O040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>C057</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>P059</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Oxfam</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Campaign 4 - General Technology Internship</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - data, IT, and technology support</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Dear Oxfam Team,
+I am a BSc Data Science student at the Open University of Kenya, expecting to graduate in 2027. I am writing to express my interest in joining your organisation for an internship or industrial attachment to support your general technology, IT, and data work.
+Through my studies and software projects, I have built practical skills in Python, R, Excel, SQL, data analysis, visualization, and basic machine learning, along with experience in web development and technical documentation. I am eager to apply these skills to support your data operations and technology needs while continuing to learn in a practical environment.
+I would like to ask whether you would consider a student intern or industrial attachment placement at this time. If you are not the correct person to speak with regarding this, could you please direct me to the appropriate team member?
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>O041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>C059</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>P060</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Mercy Corps</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Campaign 4 - General Technology Internship</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - technology, IT and data work</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Dear Mercy Corps Team,
+I am a BSc Data Science student at the Open University of Kenya, with an expected graduation year of 2027.
+I am writing to express my interest in an internship or industrial attachment focusing on general technology, IT and data work, aligned with your program monitoring, data collection, research, and digital financial inclusion initiatives such as AgriFin.
+Through my studies and personal projects, I have built skills in Python, R, Excel, SQL, data analysis, visualization, basic machine learning, and software projects. I am looking to apply these foundational technical skills in a practical environment while supporting your team.
+Would you consider an intern or industrial attachment placement for these areas, and could you direct me to the appropriate person if this is handled elsewhere?
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>O042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>C062</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>P061</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Central Bank of Kenya</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Campaign 4 - General Technology Internship</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - data, IT and technology support</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Dear Central Bank of Kenya Team,
+My name is Monica Wughanga Masae, and I am studying for a BSc in Data Science at the Open University of Kenya, with an expected graduation year of 2027.
+I am writing to enquire about internship or industrial attachment opportunities involving technology, IT, and data work, noting your functions in economic research, statistical data collection, financial datasets management, and national payments system oversight.
+Through my studies and personal projects, I have built practical skills in Python, R, SQL, Excel, data analysis, data visualization, basic machine learning, and software development, and I am available to start immediately in Nairobi. I want to contribute to your data and technology tasks while building my practical skills in a professional environment.
+Could you please let me know if you consider interns or industrial attachment students for these areas, and who the appropriate person to contact would be if not you?
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>O043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>C065</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>P063</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>The National Treasury Kenya</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Campaign 2 - Software / Technology Internship</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - software and web development support</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Dear The National Treasury Kenya Team,
+My name is Monica Wughanga Masae, and I am studying for a BSc Data Science at the Open University of Kenya, with an expected graduation year of 2027.
+I am writing to enquire about an internship or industrial attachment placement related to your management of large-scale government financial systems, public investment management platforms, and financial reporting databases.
+Through my studies and personal projects, I have built skills in Python, SQL, web development, and software projects, and I am keen to apply and grow these technical capabilities through application support and software development work.
+I would like to know if you would consider an intern or industrial attachment placement within your technology function, and who I should direct this enquiry to if you do not handle these requests directly.
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>O044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>C069</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>P065</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Kenya Power</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Campaign 2 - Software / Technology Internship</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - software and web development support</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Dear Kenya Power Team,
+I am a BSc Data Science student at the Open University of Kenya, expecting to graduate in 2027.
+I am writing to enquire about internship or industrial attachment opportunities relating to the management of customer self-service portals, digital applications like myPower, and underlying utility data systems.
+Through my coursework and software projects, I have built skills in Python, SQL, web development, and application support. I am looking for a placement where I can apply these technical skills while learning from your team.
+Could you please let me know if you would consider an intern or industrial attachment placement in these areas, and who the appropriate person to speak with would be if this is outside your remit?
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>O045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>C070</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>P066</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Wasoko</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Campaign 2 - Software / Technology Internship</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - software and web development</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Dear Wasoko Team,
+I am a student at the Open University of Kenya studying for a BSc in Data Science, with an expected graduation year of 2027.
+I am writing to enquire about internship or industrial attachment opportunities within your software development, product engineering, and digital retail operations.
+Through my studies and personal projects, I have built skills in Python, R, SQL, web development, and software projects, along with data analysis and basic machine learning. I am looking to contribute to software and web development and application support work while developing my technical skills in a professional setting.
+Could you please let me know if you consider interns or industrial attachment students for these areas, and who I might speak with if there are open positions?
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>O046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>C071</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>P067</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Pezesha</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Campaign 2 - Software / Technology Internship</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - software and web development</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Dear Pezesha Team,
+I am a BSc Data Science student at the Open University of Kenya, expecting to graduate in 2027.
+I am writing to enquire about opportunities for an internship or industrial attachment related to your work in API-driven alternative credit scoring, data point analysis, and digital loan management systems.
+Through my studies and personal projects, I have built skills in Python, R, SQL, software projects, and web development, along with basic machine learning and data analysis. I am looking for a placement where I can contribute to software and web development and application support work while developing my technical skills further.
+Could you let me know if you currently consider interns or industrial attachment students for these areas, and who the appropriate person is to speak with regarding such placements?
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>O047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>C072</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>P069</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>4G Capital</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Campaign 2 - Software / Technology Internship</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - software and web development support</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Dear 4G Capital Team,
+I am a BSc Data Science student at the Open University of Kenya, graduating in 2027.
+I am writing to enquire about opportunities at 4G Capital, which delivers smart business loans, training, and digital financial services using a fintech platform that utilizes AI to right-size loans, alongside mobile money disbursements.
+Through my studies and personal software projects, I have built skills in Python, SQL, web development, and software projects, and I am looking to contribute to software and web development and application support work while developing my technical capabilities further.
+I would like to know if you would consider an intern or industrial attachment placement in these areas, or who I should speak to if these placements are handled elsewhere.
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>O048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>C073</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>P072</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Turaco</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Campaign 4 - General Technology Internship</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Internship enquiry - data, IT, and technology support, BSc Data Science student</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Dear Turaco Team,
+I am a BSc Data Science student at the Open University of Kenya, graduating in 2027, seeking an internship or industrial attachment in Nairobi.
+I am reaching out because Turaco provides microinsurance products through partnerships with top brands and financial institutions, and develops and maintains claims and policy administration technology to support your embedded insurance services.
+Through my studies and software projects, I have built skills in Python, R, SQL, data analysis, data visualization, and basic machine learning, along with technical documentation and reporting. I want to apply these skills to support your technology, IT, and data operations while continuing to learn.
+Could you please let me know if you would consider an intern or industrial attachment placement for these functions, or direct me to the right person to speak with if not?
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>O049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>C076</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>P074</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Glovo</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Campaign 2 - Software / Technology Internship</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - software and web development support</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Dear Glovo Team,
+I am a BSc Data Science student at the Open University of Kenya, graduating in 2027.
+I am writing to enquire about internship or industrial attachment opportunities relating to your digital delivery platform and mobile application.
+Through my studies and personal projects, I have built skills in Python, R, SQL, web development, and software projects, along with data analysis and basic machine learning. I am looking to contribute to your software and web development or application support work while developing my technical skills further in a professional environment.
+Could you please let me know if you consider students for internship or industrial attachment placements, or point me to the right person to contact regarding this?
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>O050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>C077</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>P075</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Bolt</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Campaign 2 - Software / Technology Internship</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - software and web development support</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Dear Bolt Team,
+I am a student at the Open University of Kenya studying for a BSc in Data Science, with an expected graduation in 2027.
+I am reaching out regarding potential internship or industrial attachment opportunities because your technology function involves software development, data operations, and AI-powered urban mobility features.
+Through my studies and software projects, I have built skills in Python, R, SQL, and web development, alongside data analysis and reporting. I am looking to apply these technical skills and learn practical software and web development processes in a professional environment.
+Could you please let me know if you consider students for internships or industrial attachments, or direct me to the correct person to speak with regarding these roles?
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T1"/>
+  <autoFilter ref="A1:T51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10213,7 +13345,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B1"/>
+  <autoFilter ref="A1:B15"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId2"/>

</xml_diff>

<commit_message>
Add verify-sent to reconcile the workbook against Gmail
</commit_message>
<xml_diff>
--- a/data/internship_outreach.xlsx
+++ b/data/internship_outreach.xlsx
@@ -14,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Companies'!$A$1:$AA$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Contacts'!$A$1:$L$90</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Outreach'!$A$1:$T$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Outreach'!$A$1:$T$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Settings'!$A$1:$B$15</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>An international financial institution that provides loans, advice, and research to developing countries to reduce poverty and promote development.</t>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -5845,7 +5845,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>The Kenya Red Cross Society is a humanitarian relief organization that works to alleviate human suffering, manage disasters, and provide health and community services.</t>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -5948,7 +5948,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Amref Health Africa works with communities and governments to strengthen health systems and advance African-led health solutions.</t>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>PATH transforms innovative ideas into global health breakthroughs, operating in over 70 countries including Kenya.</t>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -6154,7 +6154,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Population Services International is a global network of locally-led organizations focused on transforming health by tackling root causes and delivering healthcare products and services.</t>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -6257,7 +6257,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>CARE International is an international humanitarian aid and development organization dedicated to ending poverty and providing emergency support.</t>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -15138,7 +15138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T51"/>
+  <dimension ref="A1:T57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="3"/>
@@ -15272,7 +15272,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>P001</t>
+          <t>P002</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -15505,7 +15505,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>P025</t>
+          <t>P026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -15654,7 +15654,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>P007</t>
+          <t>P008</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -15700,7 +15700,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -15708,9 +15708,19 @@
           <t>2026-09-14</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P7" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a48cb0ce8936a</t>
         </is>
       </c>
     </row>
@@ -16233,7 +16243,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>P016</t>
+          <t>P017</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -16532,7 +16542,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>P025</t>
+          <t>P026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -16609,7 +16619,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>P027</t>
+          <t>P046</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -16682,7 +16692,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>P028</t>
+          <t>P029</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -16727,7 +16737,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -16735,9 +16745,19 @@
           <t>2026-09-14</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P21" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a48d281f42132</t>
         </is>
       </c>
     </row>
@@ -16836,7 +16856,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>P034</t>
+          <t>P035</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -16881,7 +16901,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -16889,9 +16909,19 @@
           <t>2026-09-14</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P23" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a48da081ed55d</t>
         </is>
       </c>
     </row>
@@ -17341,7 +17371,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>P048</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -17418,7 +17448,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>P046</t>
+          <t>P048</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -17495,7 +17525,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>P047</t>
+          <t>P049</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -17567,7 +17597,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>P048</t>
+          <t>P051</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -17613,7 +17643,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -17621,9 +17651,19 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P33" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a48e18f293966</t>
         </is>
       </c>
     </row>
@@ -17640,7 +17680,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>P049</t>
+          <t>P053</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -17712,7 +17752,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>P050</t>
+          <t>P055</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -17757,7 +17797,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -17765,9 +17805,19 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P35" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a48e910ff70fe</t>
         </is>
       </c>
     </row>
@@ -17784,7 +17834,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>P051</t>
+          <t>P057</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -17857,7 +17907,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>P052</t>
+          <t>P059</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -17903,7 +17953,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -17911,9 +17961,19 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P37" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a4940b8d1ce3b</t>
         </is>
       </c>
     </row>
@@ -17930,7 +17990,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>P054</t>
+          <t>P061</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -17975,7 +18035,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -17983,9 +18043,19 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P38" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a4948368bdeba</t>
         </is>
       </c>
     </row>
@@ -18002,7 +18072,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>P056</t>
+          <t>P062</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -18074,7 +18144,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>P057</t>
+          <t>P064</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -18119,7 +18189,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -18127,9 +18197,19 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P40" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a494fca1bda15</t>
         </is>
       </c>
     </row>
@@ -18146,7 +18226,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>P059</t>
+          <t>P065</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -18218,7 +18298,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>P060</t>
+          <t>P066</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -18290,7 +18370,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>P061</t>
+          <t>P068</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -18335,7 +18415,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -18343,9 +18423,19 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P43" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a4957571902b0</t>
         </is>
       </c>
     </row>
@@ -18362,7 +18452,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>P063</t>
+          <t>P070</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -18408,7 +18498,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -18416,9 +18506,19 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P44" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a495ecf76000d</t>
         </is>
       </c>
     </row>
@@ -18435,7 +18535,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>P065</t>
+          <t>P071</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -18481,7 +18581,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -18489,9 +18589,19 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P45" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a49a5ce9ea91c</t>
         </is>
       </c>
     </row>
@@ -18508,7 +18618,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>P066</t>
+          <t>P072</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -18580,7 +18690,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>P067</t>
+          <t>P074</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -18626,7 +18736,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -18634,9 +18744,19 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P47" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a49ad527e0f24</t>
         </is>
       </c>
     </row>
@@ -18653,7 +18773,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>P069</t>
+          <t>P076</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -18698,7 +18818,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -18706,9 +18826,19 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P48" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a49b4c026b921</t>
         </is>
       </c>
     </row>
@@ -18725,7 +18855,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>P072</t>
+          <t>P079</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -18771,7 +18901,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>DRAFTED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -18779,9 +18909,19 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
       <c r="P49" t="inlineStr">
         <is>
           <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a49bc444ffadf</t>
         </is>
       </c>
     </row>
@@ -18798,7 +18938,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>P074</t>
+          <t>P081</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -18871,7 +19011,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>P075</t>
+          <t>P084</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -18931,8 +19071,454 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>O051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>C074</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>P080</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Jumia Kenya</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Campaign 2 - Software / Technology Internship</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Industrial attachment enquiry - software and web development</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Dear Jumia Kenya Team,
+I am Monica Wughanga Masae, a BSc Data Science student at the Open University of Kenya, graduating in 2027.
+I am writing to express my interest in an internship or industrial attachment focusing on software and web development, and application support work, given that you operate an online e-commerce marketplace and retail platform involving e-commerce platform development and web and application operations.
+Through my studies and personal work, I have built skills in Python, R, SQL, web development, and software projects, along with data analysis and reporting. I am looking to contribute to your technology operations while gaining practical experience.
+Could you please let me know if you consider students for an industrial attachment or internship placement in these areas, and who the appropriate person to speak with would be if this is outside your remit?
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>O052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>C017</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>P082</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>JamboPay</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Campaign 1 - Data / Analytics Internship</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Internship enquiry - data analysis and reporting, BSc Data Science student</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Dear JamboPay Team,
+I am a student at the Open University of Kenya pursuing a BSc in Data Science, with an expected graduation year of 2027.
+I am reaching out regarding internship and industrial attachment opportunities because of your work providing regulated payment gateway, checkout APIs, and financial transaction infrastructure.
+Through my studies and projects, I have built practical skills in Python, R, SQL, Excel, data analysis, and data visualization using tools like Tableau. I am looking for a placement where I can contribute to data analysis, reporting, and visualization work while learning from your team.
+Could you let me know if you consider interns or industrial attachment students, and who the appropriate person is to speak with regarding these opportunities?
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>O053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>C045</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>P083</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>BETA Agriculture Technologies</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Campaign 1 - Data / Analytics Internship</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Internship enquiry - data analysis, BSc Data Science student</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Dear BETA Agriculture Technologies Team,
+I am a BSc Data Science student at the Open University of Kenya, expecting to graduate in 2027.
+I am writing to enquire about internship or industrial attachment opportunities relating to the digital solutions powered by AI, IoT, satellite monitoring, and precision farming technologies that you provide for farmers, agribusinesses, and financial institutions in East Africa.
+Through my studies and software projects, I have built practical skills in data analysis, reporting, data visualization, Python, R, SQL, and Excel. I am looking for a placement where I can contribute to data analysis and reporting work while learning from your deployment of AI-powered agronomy, satellite monitoring, IoT smart sensors, and data analytics for agriculture.
+Could you please let me know if you would consider an intern or industrial attachment placement, and who I should speak with if you are not the correct contact?
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>O054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>C078</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>P085</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Ackyshine Monitoring and Evaluation Consultancy</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Campaign 1 - Data / Analytics Internship</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Internship enquiry - data analysis and reporting, BSc Data Science student</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Dear Ackyshine Monitoring and Evaluation Consultancy Team,
+I am Monica Wughanga Masae, a BSc Data Science student at the Open University of Kenya graduating in 2027.
+I am writing to enquire about potential internship or industrial attachment opportunities relating to your AI-integrated digital platform, which involves data dashboards, modules, and AI support.
+Through my studies and personal projects, I have built practical skills in Python, R, SQL, and Excel. My strongest area is data analysis, reporting, and visualization, supported by exposure to Tableau, basic statistics, and software projects. I am eager to contribute to your data analysis and reporting tasks while further developing my technical skills.
+Could you please let me know if you would consider an intern or industrial attachment placement for this type of work, or direct me to the right person to speak with if you handle these enquiries elsewhere?
+Thank you for your time.
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>O055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>C083</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>P086</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Third Party Monitoring and Evaluation Limited</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Campaign 1 - Data / Analytics Internship</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Internship enquiry - data analysis, reporting and visualisation</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Dear Third Party Monitoring and Evaluation Limited Team,
+My name is Monica Wughanga Masae, and I am studying BSc Data Science at the Open University of Kenya, with an expected graduation year of 2027.
+I am reaching out because Third Party Monitoring and Evaluation Limited provides project monitoring, evaluation, learning, research, and data analytics services, with a technology function that includes data analytics, data visualizations, M&amp;E systems, automated research tools coding, and cloud data hosting.
+Through my studies, I have built skills in data analysis, reporting, data visualization, Python, R, Excel, SQL, and Tableau exposure. I want to apply these skills to support your data analysis, reporting, and visualisation work while learning practical workflows in an organisation focused on research and data analytics.
+I am writing to ask whether you would consider a student for an internship or industrial attachment placement, and who I should speak with if you accept applications for these roles.
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>DRAFTED</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>O056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>C085</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>P087</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>MNC Consulting</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Campaign 1 - Data / Analytics Internship</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Internship enquiry - data analysis and reporting, BSc Data Science student</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Dear MNC Consulting Team,
+I am Monica Wughanga Masae, a BSc Data Science student at the Open University of Kenya, graduating in 2027. I am writing to enquire about an internship or industrial attachment.
+I am interested in your work in communication services such as USSD and Bulk SMS, as well as digital HR modules including HR Analytics.
+Through my studies and personal projects, I have built skills in Python, R, SQL, Excel, data analysis, reporting, and data visualization. I am looking to contribute to your data analysis, reporting, and visualization work while learning practical operations in a professional setting.
+Could you please let me know if you consider interns or industrial attachment students, and who I should direct my application to if appropriate?
+Thank you for your time.
+Kind regards,
+Monica Wughanga Masae
+BSc Data Science, Open University of Kenya (expected 2027)
+monicawughanga@gmail.com
+LinkedIn: https://www.linkedin.com/in/monica-masae/
+GitHub: https://github.com/M0nicah</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Gmail message id: 1a0a4af713ed128b</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T51"/>
+  <autoFilter ref="A1:T57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>